<commit_message>
Tuning values n things
</commit_message>
<xml_diff>
--- a/hsv_color_data.xlsx
+++ b/hsv_color_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,365 +447,420 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>62</v>
+        <v>114</v>
       </c>
       <c r="B2" t="n">
-        <v>161</v>
+        <v>216</v>
       </c>
       <c r="C2" t="n">
-        <v>204</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="B3" t="n">
+        <v>202</v>
+      </c>
+      <c r="C3" t="n">
         <v>160</v>
-      </c>
-      <c r="C3" t="n">
-        <v>206</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="B4" t="n">
-        <v>155</v>
+        <v>187</v>
       </c>
       <c r="C4" t="n">
-        <v>209</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>62</v>
+        <v>112</v>
       </c>
       <c r="B5" t="n">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="C5" t="n">
-        <v>171</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>66</v>
+        <v>113</v>
       </c>
       <c r="B6" t="n">
-        <v>197</v>
+        <v>234</v>
       </c>
       <c r="C6" t="n">
-        <v>179</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="B7" t="n">
-        <v>148</v>
+        <v>208</v>
       </c>
       <c r="C7" t="n">
-        <v>213</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="B8" t="n">
-        <v>153</v>
+        <v>187</v>
       </c>
       <c r="C8" t="n">
-        <v>211</v>
+        <v>173</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>63</v>
+        <v>111</v>
       </c>
       <c r="B9" t="n">
-        <v>160</v>
+        <v>192</v>
       </c>
       <c r="C9" t="n">
-        <v>201</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="B10" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C10" t="n">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>62</v>
+        <v>115</v>
       </c>
       <c r="B11" t="n">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="C11" t="n">
-        <v>219</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>61</v>
+        <v>114</v>
       </c>
       <c r="B12" t="n">
-        <v>153</v>
+        <v>180</v>
       </c>
       <c r="C12" t="n">
-        <v>211</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="B13" t="n">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="C13" t="n">
-        <v>255</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>57</v>
+        <v>114</v>
       </c>
       <c r="B14" t="n">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="C14" t="n">
-        <v>255</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>62</v>
+        <v>101</v>
       </c>
       <c r="B15" t="n">
-        <v>146</v>
+        <v>174</v>
       </c>
       <c r="C15" t="n">
-        <v>243</v>
+        <v>193</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="B16" t="n">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="C16" t="n">
-        <v>238</v>
+        <v>172</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="B17" t="n">
-        <v>136</v>
+        <v>162</v>
       </c>
       <c r="C17" t="n">
-        <v>249</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="B18" t="n">
-        <v>132</v>
+        <v>176</v>
       </c>
       <c r="C18" t="n">
-        <v>255</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>61</v>
+        <v>109</v>
       </c>
       <c r="B19" t="n">
-        <v>128</v>
+        <v>175</v>
       </c>
       <c r="C19" t="n">
-        <v>255</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>61</v>
+        <v>108</v>
       </c>
       <c r="B20" t="n">
-        <v>139</v>
+        <v>192</v>
       </c>
       <c r="C20" t="n">
-        <v>243</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="B21" t="n">
-        <v>134</v>
+        <v>197</v>
       </c>
       <c r="C21" t="n">
-        <v>255</v>
+        <v>192</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>63</v>
+        <v>115</v>
       </c>
       <c r="B22" t="n">
-        <v>148</v>
+        <v>182</v>
       </c>
       <c r="C22" t="n">
-        <v>255</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="B23" t="n">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="C23" t="n">
-        <v>255</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>62</v>
+        <v>110</v>
       </c>
       <c r="B24" t="n">
-        <v>162</v>
+        <v>186</v>
       </c>
       <c r="C24" t="n">
-        <v>248</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>61</v>
+        <v>113</v>
       </c>
       <c r="B25" t="n">
-        <v>147</v>
+        <v>204</v>
       </c>
       <c r="C25" t="n">
-        <v>241</v>
+        <v>201</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="B26" t="n">
-        <v>150</v>
+        <v>197</v>
       </c>
       <c r="C26" t="n">
-        <v>233</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="B27" t="n">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="C27" t="n">
-        <v>246</v>
+        <v>167</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="B28" t="n">
+        <v>174</v>
+      </c>
+      <c r="C28" t="n">
         <v>135</v>
-      </c>
-      <c r="C28" t="n">
-        <v>241</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="B29" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C29" t="n">
-        <v>255</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="B30" t="n">
-        <v>152</v>
+        <v>207</v>
       </c>
       <c r="C30" t="n">
-        <v>210</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="B31" t="n">
-        <v>143</v>
+        <v>220</v>
       </c>
       <c r="C31" t="n">
-        <v>201</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>63</v>
+        <v>112</v>
       </c>
       <c r="B32" t="n">
-        <v>142</v>
+        <v>238</v>
       </c>
       <c r="C32" t="n">
-        <v>255</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="B33" t="n">
-        <v>124</v>
+        <v>255</v>
       </c>
       <c r="C33" t="n">
-        <v>255</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>63</v>
+        <v>112</v>
       </c>
       <c r="B34" t="n">
+        <v>215</v>
+      </c>
+      <c r="C34" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>112</v>
+      </c>
+      <c r="B35" t="n">
+        <v>191</v>
+      </c>
+      <c r="C35" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>113</v>
+      </c>
+      <c r="B36" t="n">
+        <v>177</v>
+      </c>
+      <c r="C36" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>112</v>
+      </c>
+      <c r="B37" t="n">
+        <v>190</v>
+      </c>
+      <c r="C37" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>113</v>
+      </c>
+      <c r="B38" t="n">
+        <v>188</v>
+      </c>
+      <c r="C38" t="n">
         <v>167</v>
       </c>
-      <c r="C34" t="n">
-        <v>215</v>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>111</v>
+      </c>
+      <c r="B39" t="n">
+        <v>118</v>
+      </c>
+      <c r="C39" t="n">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>